<commit_message>
baremo correction and getting age from register
</commit_message>
<xml_diff>
--- a/Baremo.xlsx
+++ b/Baremo.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/luli/Desktop/StroopTest/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/luli/Desktop/Cognitio/StroopTest/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D25BAE6-E554-7D4F-B667-2B6800358144}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCB408F3-DBD1-D943-B5BB-018B5B70D95E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6440" yWindow="760" windowWidth="25660" windowHeight="15820" activeTab="1" xr2:uid="{02CFBACB-F405-5C48-87EF-3F16FF9EFC01}"/>
+    <workbookView xWindow="13520" yWindow="0" windowWidth="14000" windowHeight="15820" xr2:uid="{02CFBACB-F405-5C48-87EF-3F16FF9EFC01}"/>
   </bookViews>
   <sheets>
     <sheet name="P" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="PC" sheetId="3" r:id="rId3"/>
     <sheet name="I" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -462,7 +462,7 @@
         <v>165</v>
       </c>
       <c r="B5">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
@@ -494,7 +494,7 @@
         <v>161</v>
       </c>
       <c r="B9">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
@@ -526,7 +526,7 @@
         <v>157</v>
       </c>
       <c r="B13">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
@@ -558,7 +558,7 @@
         <v>153</v>
       </c>
       <c r="B17">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
@@ -590,7 +590,7 @@
         <v>149</v>
       </c>
       <c r="B21">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
@@ -622,7 +622,7 @@
         <v>145</v>
       </c>
       <c r="B25">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
@@ -654,7 +654,7 @@
         <v>141</v>
       </c>
       <c r="B29">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
@@ -686,7 +686,7 @@
         <v>137</v>
       </c>
       <c r="B33">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.2">
@@ -718,7 +718,7 @@
         <v>133</v>
       </c>
       <c r="B37">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.2">
@@ -750,7 +750,7 @@
         <v>129</v>
       </c>
       <c r="B41">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.2">
@@ -782,7 +782,7 @@
         <v>125</v>
       </c>
       <c r="B45">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.2">
@@ -814,7 +814,7 @@
         <v>121</v>
       </c>
       <c r="B49">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.2">
@@ -846,7 +846,7 @@
         <v>117</v>
       </c>
       <c r="B53">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.2">
@@ -878,7 +878,7 @@
         <v>113</v>
       </c>
       <c r="B57">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.2">
@@ -910,7 +910,7 @@
         <v>109</v>
       </c>
       <c r="B61">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.2">
@@ -942,7 +942,7 @@
         <v>105</v>
       </c>
       <c r="B65">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.2">
@@ -974,7 +974,7 @@
         <v>101</v>
       </c>
       <c r="B69">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.2">
@@ -1006,7 +1006,7 @@
         <v>97</v>
       </c>
       <c r="B73">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.2">
@@ -1038,7 +1038,7 @@
         <v>93</v>
       </c>
       <c r="B77">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.2">
@@ -1070,7 +1070,7 @@
         <v>89</v>
       </c>
       <c r="B81">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.2">
@@ -1102,7 +1102,7 @@
         <v>85</v>
       </c>
       <c r="B85">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.2">
@@ -1134,7 +1134,7 @@
         <v>81</v>
       </c>
       <c r="B89">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.2">
@@ -1166,7 +1166,7 @@
         <v>77</v>
       </c>
       <c r="B93">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.2">
@@ -1198,7 +1198,7 @@
         <v>73</v>
       </c>
       <c r="B97">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="98" spans="1:2" x14ac:dyDescent="0.2">
@@ -1230,7 +1230,7 @@
         <v>69</v>
       </c>
       <c r="B101">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="102" spans="1:2" x14ac:dyDescent="0.2">
@@ -1262,7 +1262,7 @@
         <v>65</v>
       </c>
       <c r="B105">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="106" spans="1:2" x14ac:dyDescent="0.2">
@@ -1294,7 +1294,7 @@
         <v>61</v>
       </c>
       <c r="B109">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="110" spans="1:2" x14ac:dyDescent="0.2">
@@ -1326,7 +1326,7 @@
         <v>57</v>
       </c>
       <c r="B113">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="114" spans="1:2" x14ac:dyDescent="0.2">
@@ -1358,7 +1358,7 @@
         <v>53</v>
       </c>
       <c r="B117">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="118" spans="1:2" x14ac:dyDescent="0.2">
@@ -1390,7 +1390,7 @@
         <v>49</v>
       </c>
       <c r="B121">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="122" spans="1:2" x14ac:dyDescent="0.2">
@@ -1440,7 +1440,7 @@
         <v>123</v>
       </c>
       <c r="B4">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
@@ -1464,7 +1464,7 @@
         <v>120</v>
       </c>
       <c r="B7">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
@@ -1488,7 +1488,7 @@
         <v>117</v>
       </c>
       <c r="B10">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
@@ -1512,7 +1512,7 @@
         <v>114</v>
       </c>
       <c r="B13">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
@@ -1536,7 +1536,7 @@
         <v>111</v>
       </c>
       <c r="B16">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
@@ -1560,7 +1560,7 @@
         <v>108</v>
       </c>
       <c r="B19">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
@@ -1584,7 +1584,7 @@
         <v>105</v>
       </c>
       <c r="B22">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
@@ -1608,7 +1608,7 @@
         <v>102</v>
       </c>
       <c r="B25">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
@@ -1632,7 +1632,7 @@
         <v>99</v>
       </c>
       <c r="B28">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
@@ -1656,7 +1656,7 @@
         <v>96</v>
       </c>
       <c r="B31">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
@@ -1680,7 +1680,7 @@
         <v>93</v>
       </c>
       <c r="B34">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.2">
@@ -1704,7 +1704,7 @@
         <v>90</v>
       </c>
       <c r="B37">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.2">
@@ -1728,7 +1728,7 @@
         <v>87</v>
       </c>
       <c r="B40">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.2">
@@ -1752,7 +1752,7 @@
         <v>84</v>
       </c>
       <c r="B43">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.2">
@@ -1776,7 +1776,7 @@
         <v>81</v>
       </c>
       <c r="B46">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.2">
@@ -1800,7 +1800,7 @@
         <v>78</v>
       </c>
       <c r="B49">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.2">
@@ -1824,7 +1824,7 @@
         <v>75</v>
       </c>
       <c r="B52">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.2">
@@ -1848,7 +1848,7 @@
         <v>72</v>
       </c>
       <c r="B55">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.2">
@@ -1872,7 +1872,7 @@
         <v>69</v>
       </c>
       <c r="B58">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.2">
@@ -1896,7 +1896,7 @@
         <v>66</v>
       </c>
       <c r="B61">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.2">
@@ -1920,7 +1920,7 @@
         <v>63</v>
       </c>
       <c r="B64">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.2">
@@ -1944,7 +1944,7 @@
         <v>60</v>
       </c>
       <c r="B67">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.2">
@@ -1968,7 +1968,7 @@
         <v>57</v>
       </c>
       <c r="B70">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.2">
@@ -1992,7 +1992,7 @@
         <v>54</v>
       </c>
       <c r="B73">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.2">
@@ -2016,7 +2016,7 @@
         <v>51</v>
       </c>
       <c r="B76">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.2">
@@ -2040,7 +2040,7 @@
         <v>48</v>
       </c>
       <c r="B79">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.2">
@@ -2064,7 +2064,7 @@
         <v>45</v>
       </c>
       <c r="B82">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.2">
@@ -2088,7 +2088,7 @@
         <v>42</v>
       </c>
       <c r="B85">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.2">
@@ -2112,7 +2112,7 @@
         <v>39</v>
       </c>
       <c r="B88">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.2">
@@ -2136,7 +2136,7 @@
         <v>36</v>
       </c>
       <c r="B91">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.2">

</xml_diff>